<commit_message>
having a hard time pulling myself away from this. Must stop now.
</commit_message>
<xml_diff>
--- a/Spreadsheets/Parts_HVPSController2.xlsx
+++ b/Spreadsheets/Parts_HVPSController2.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1896" uniqueCount="630">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1899" uniqueCount="631">
   <si>
     <t>Item #</t>
   </si>
@@ -1915,6 +1915,9 @@
   </si>
   <si>
     <t>[?]</t>
+  </si>
+  <si>
+    <t>4.7nF</t>
   </si>
 </sst>
 </file>
@@ -6400,7 +6403,9 @@
       <c r="I49" s="27"/>
       <c r="J49" s="28"/>
       <c r="K49" s="29"/>
-      <c r="L49" s="30"/>
+      <c r="L49" s="30" t="s">
+        <v>630</v>
+      </c>
       <c r="M49" s="31"/>
       <c r="N49" s="32"/>
       <c r="O49" s="24"/>
@@ -8616,7 +8621,7 @@
         <v>314</v>
       </c>
       <c r="C104" s="33" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D104" s="49" t="s">
         <v>521</v>
@@ -8661,7 +8666,7 @@
         <v>315</v>
       </c>
       <c r="C105" s="33" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D105" s="49" t="s">
         <v>521</v>
@@ -8704,7 +8709,9 @@
       <c r="B106" s="151" t="s">
         <v>316</v>
       </c>
-      <c r="C106" s="33"/>
+      <c r="C106" s="33" t="s">
+        <v>628</v>
+      </c>
       <c r="D106" s="49" t="s">
         <v>524</v>
       </c>
@@ -8746,7 +8753,9 @@
       <c r="B107" s="151" t="s">
         <v>317</v>
       </c>
-      <c r="C107" s="33"/>
+      <c r="C107" s="33" t="s">
+        <v>629</v>
+      </c>
       <c r="D107" s="49" t="s">
         <v>528</v>
       </c>
@@ -8915,7 +8924,7 @@
         <v>322</v>
       </c>
       <c r="C112" s="33" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D112" s="49" t="s">
         <v>521</v>
@@ -9061,7 +9070,7 @@
         <v>325</v>
       </c>
       <c r="C116" s="33" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D116" s="49" t="s">
         <v>521</v>
@@ -9105,7 +9114,7 @@
         <v>326</v>
       </c>
       <c r="C117" s="33" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D117" s="49" t="s">
         <v>521</v>
@@ -9149,7 +9158,7 @@
         <v>327</v>
       </c>
       <c r="C118" s="33" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D118" s="49" t="s">
         <v>521</v>
@@ -9671,7 +9680,7 @@
         <v>343</v>
       </c>
       <c r="C134" s="33" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D134" s="142" t="s">
         <v>473</v>
@@ -9713,7 +9722,7 @@
         <v>344</v>
       </c>
       <c r="C135" s="33" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D135" s="142" t="s">
         <v>473</v>
@@ -9755,7 +9764,7 @@
         <v>345</v>
       </c>
       <c r="C136" s="33" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D136" s="142" t="s">
         <v>473</v>
@@ -11587,7 +11596,7 @@
         <v>393</v>
       </c>
       <c r="C184" s="33" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D184" s="142" t="s">
         <v>581</v>
@@ -11903,7 +11912,7 @@
         <v>399</v>
       </c>
       <c r="C192" s="33" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D192" s="142" t="s">
         <v>596</v>
@@ -12025,7 +12034,7 @@
         <v>402</v>
       </c>
       <c r="C195" s="33" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D195" s="142" t="s">
         <v>596</v>
@@ -12547,7 +12556,7 @@
         <v>415</v>
       </c>
       <c r="C208" s="33" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D208" s="142" t="s">
         <v>596</v>
@@ -21253,9 +21262,10 @@
     <hyperlink ref="D216" r:id="rId71"/>
     <hyperlink ref="D212" r:id="rId72"/>
     <hyperlink ref="D213" r:id="rId73"/>
+    <hyperlink ref="D52" r:id="rId74"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId74"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId75"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
PCB coming together :)
</commit_message>
<xml_diff>
--- a/Spreadsheets/Parts_HVPSController2.xlsx
+++ b/Spreadsheets/Parts_HVPSController2.xlsx
@@ -1743,12 +1743,6 @@
     <t>100Ω</t>
   </si>
   <si>
-    <t>Generic 6.2 0.25w resistor</t>
-  </si>
-  <si>
-    <t>6.2Ω</t>
-  </si>
-  <si>
     <t>RV4</t>
   </si>
   <si>
@@ -1918,6 +1912,12 @@
   </si>
   <si>
     <t>4.7nF</t>
+  </si>
+  <si>
+    <t>Generic 4.7 0.25w resistor</t>
+  </si>
+  <si>
+    <t>4.7Ω</t>
   </si>
 </sst>
 </file>
@@ -4122,7 +4122,7 @@
         <v>213</v>
       </c>
       <c r="C1" s="179" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="D1" s="56" t="s">
         <v>22</v>
@@ -6404,7 +6404,7 @@
       <c r="J49" s="28"/>
       <c r="K49" s="29"/>
       <c r="L49" s="30" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="M49" s="31"/>
       <c r="N49" s="32"/>
@@ -8501,26 +8501,26 @@
     <row r="101" spans="1:23" s="141" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A101" s="166"/>
       <c r="B101" s="151" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="C101" s="33" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="D101" s="49" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="E101" s="47"/>
       <c r="F101" s="156" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="G101" s="25" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="H101" s="26"/>
       <c r="I101" s="27"/>
       <c r="J101" s="28"/>
       <c r="K101" s="29" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="L101" s="30"/>
       <c r="M101" s="40"/>
@@ -8540,26 +8540,26 @@
     <row r="102" spans="1:23" s="141" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A102" s="166"/>
       <c r="B102" s="151" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="C102" s="33" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="D102" s="49" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="E102" s="47"/>
       <c r="F102" s="156" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="G102" s="25" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="H102" s="26"/>
       <c r="I102" s="27"/>
       <c r="J102" s="28"/>
       <c r="K102" s="29" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="L102" s="30"/>
       <c r="M102" s="40"/>
@@ -8579,26 +8579,26 @@
     <row r="103" spans="1:23" s="141" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A103" s="166"/>
       <c r="B103" s="151" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="C103" s="33" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="D103" s="49" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="E103" s="47"/>
       <c r="F103" s="156" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="G103" s="25" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="H103" s="26"/>
       <c r="I103" s="27"/>
       <c r="J103" s="28"/>
       <c r="K103" s="29" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="L103" s="30"/>
       <c r="M103" s="40"/>
@@ -8621,7 +8621,7 @@
         <v>314</v>
       </c>
       <c r="C104" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D104" s="49" t="s">
         <v>521</v>
@@ -8666,7 +8666,7 @@
         <v>315</v>
       </c>
       <c r="C105" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D105" s="49" t="s">
         <v>521</v>
@@ -8710,7 +8710,7 @@
         <v>316</v>
       </c>
       <c r="C106" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D106" s="49" t="s">
         <v>524</v>
@@ -8754,7 +8754,7 @@
         <v>317</v>
       </c>
       <c r="C107" s="33" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="D107" s="49" t="s">
         <v>528</v>
@@ -8924,7 +8924,7 @@
         <v>322</v>
       </c>
       <c r="C112" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D112" s="49" t="s">
         <v>521</v>
@@ -8994,7 +8994,7 @@
         <v>313</v>
       </c>
       <c r="C114" s="33" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="D114" s="49" t="s">
         <v>530</v>
@@ -9032,7 +9032,7 @@
         <v>324</v>
       </c>
       <c r="C115" s="33" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="D115" s="49" t="s">
         <v>530</v>
@@ -9070,7 +9070,7 @@
         <v>325</v>
       </c>
       <c r="C116" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D116" s="49" t="s">
         <v>521</v>
@@ -9114,7 +9114,7 @@
         <v>326</v>
       </c>
       <c r="C117" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D117" s="49" t="s">
         <v>521</v>
@@ -9158,7 +9158,7 @@
         <v>327</v>
       </c>
       <c r="C118" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D118" s="49" t="s">
         <v>521</v>
@@ -9228,7 +9228,7 @@
         <v>329</v>
       </c>
       <c r="C120" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D120" s="49" t="s">
         <v>530</v>
@@ -9604,7 +9604,7 @@
         <v>341</v>
       </c>
       <c r="C132" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D132" s="142"/>
       <c r="E132" s="47"/>
@@ -9680,7 +9680,7 @@
         <v>343</v>
       </c>
       <c r="C134" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D134" s="142" t="s">
         <v>473</v>
@@ -9722,7 +9722,7 @@
         <v>344</v>
       </c>
       <c r="C135" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D135" s="142" t="s">
         <v>473</v>
@@ -9764,7 +9764,7 @@
         <v>345</v>
       </c>
       <c r="C136" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D136" s="142" t="s">
         <v>473</v>
@@ -9806,7 +9806,7 @@
         <v>346</v>
       </c>
       <c r="C137" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D137" s="142"/>
       <c r="E137" s="47"/>
@@ -9840,7 +9840,7 @@
         <v>347</v>
       </c>
       <c r="C138" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D138" s="142"/>
       <c r="E138" s="47"/>
@@ -9874,7 +9874,7 @@
         <v>348</v>
       </c>
       <c r="C139" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D139" s="142"/>
       <c r="E139" s="47"/>
@@ -9908,7 +9908,7 @@
         <v>349</v>
       </c>
       <c r="C140" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D140" s="142"/>
       <c r="E140" s="47"/>
@@ -9942,7 +9942,7 @@
         <v>350</v>
       </c>
       <c r="C141" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D141" s="142"/>
       <c r="E141" s="47"/>
@@ -9976,7 +9976,7 @@
         <v>351</v>
       </c>
       <c r="C142" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D142" s="142"/>
       <c r="E142" s="47"/>
@@ -10010,7 +10010,7 @@
         <v>352</v>
       </c>
       <c r="C143" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D143" s="142"/>
       <c r="E143" s="47"/>
@@ -10044,7 +10044,7 @@
         <v>353</v>
       </c>
       <c r="C144" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D144" s="142"/>
       <c r="E144" s="47"/>
@@ -10078,7 +10078,7 @@
         <v>354</v>
       </c>
       <c r="C145" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D145" s="142"/>
       <c r="E145" s="47"/>
@@ -10112,7 +10112,7 @@
         <v>355</v>
       </c>
       <c r="C146" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D146" s="142"/>
       <c r="E146" s="47"/>
@@ -10146,7 +10146,7 @@
         <v>356</v>
       </c>
       <c r="C147" s="33" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="D147" s="49" t="s">
         <v>428</v>
@@ -10976,10 +10976,10 @@
       <c r="I167" s="27"/>
       <c r="J167" s="28"/>
       <c r="K167" s="29" t="s">
-        <v>572</v>
+        <v>629</v>
       </c>
       <c r="L167" s="30" t="s">
-        <v>573</v>
+        <v>630</v>
       </c>
       <c r="M167" s="40">
         <v>0.01</v>
@@ -11016,10 +11016,10 @@
       <c r="I168" s="27"/>
       <c r="J168" s="28"/>
       <c r="K168" s="29" t="s">
-        <v>572</v>
+        <v>629</v>
       </c>
       <c r="L168" s="30" t="s">
-        <v>573</v>
+        <v>630</v>
       </c>
       <c r="M168" s="40">
         <v>0.01</v>
@@ -11312,10 +11312,10 @@
       <c r="I176" s="27"/>
       <c r="J176" s="28"/>
       <c r="K176" s="29" t="s">
-        <v>572</v>
+        <v>629</v>
       </c>
       <c r="L176" s="30" t="s">
-        <v>573</v>
+        <v>630</v>
       </c>
       <c r="M176" s="40">
         <v>0.01</v>
@@ -11352,10 +11352,10 @@
       <c r="I177" s="27"/>
       <c r="J177" s="28"/>
       <c r="K177" s="29" t="s">
-        <v>572</v>
+        <v>629</v>
       </c>
       <c r="L177" s="30" t="s">
-        <v>573</v>
+        <v>630</v>
       </c>
       <c r="M177" s="40">
         <v>0.01</v>
@@ -11519,26 +11519,26 @@
       <c r="D182" s="142"/>
       <c r="E182" s="47"/>
       <c r="F182" s="24" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="G182" s="25" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="H182" s="26"/>
       <c r="I182" s="27"/>
       <c r="J182" s="28"/>
       <c r="K182" s="29" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="L182" s="30" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="M182" s="40">
         <v>0.1</v>
       </c>
       <c r="N182" s="32"/>
       <c r="O182" s="24" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="P182" s="33"/>
       <c r="Q182" s="34" t="s">
@@ -11559,16 +11559,16 @@
       <c r="D183" s="142"/>
       <c r="E183" s="47"/>
       <c r="F183" s="24" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="G183" s="25" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="H183" s="26"/>
       <c r="I183" s="27"/>
       <c r="J183" s="28"/>
       <c r="K183" s="29" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="L183" s="30" t="s">
         <v>563</v>
@@ -11578,7 +11578,7 @@
       </c>
       <c r="N183" s="32"/>
       <c r="O183" s="24" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="P183" s="33"/>
       <c r="Q183" s="34" t="s">
@@ -11596,33 +11596,33 @@
         <v>393</v>
       </c>
       <c r="C184" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D184" s="142" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="E184" s="47"/>
       <c r="F184" s="24" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="G184" s="25" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="H184" s="26"/>
       <c r="I184" s="27"/>
       <c r="J184" s="28"/>
       <c r="K184" s="29" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="L184" s="30" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="M184" s="40">
         <v>0.1</v>
       </c>
       <c r="N184" s="32"/>
       <c r="O184" s="24" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="P184" s="33"/>
       <c r="Q184" s="34" t="s">
@@ -11637,22 +11637,22 @@
     <row r="185" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A185" s="166"/>
       <c r="B185" s="148" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="C185" s="33"/>
       <c r="D185" s="142"/>
       <c r="E185" s="47"/>
       <c r="F185" s="24" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="G185" s="25" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="H185" s="26"/>
       <c r="I185" s="27"/>
       <c r="J185" s="28"/>
       <c r="K185" s="29" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="L185" s="30" t="s">
         <v>563</v>
@@ -11662,7 +11662,7 @@
       </c>
       <c r="N185" s="32"/>
       <c r="O185" s="24" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="P185" s="33"/>
       <c r="Q185" s="34" t="s">
@@ -11677,32 +11677,32 @@
     <row r="186" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A186" s="166"/>
       <c r="B186" s="148" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="C186" s="33"/>
       <c r="D186" s="142"/>
       <c r="E186" s="47"/>
       <c r="F186" s="24" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="G186" s="25" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="H186" s="26"/>
       <c r="I186" s="27"/>
       <c r="J186" s="28"/>
       <c r="K186" s="29" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="L186" s="30" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="M186" s="40">
         <v>0.1</v>
       </c>
       <c r="N186" s="32"/>
       <c r="O186" s="24" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="P186" s="33"/>
       <c r="Q186" s="34" t="s">
@@ -11721,20 +11721,20 @@
       </c>
       <c r="C187" s="33"/>
       <c r="D187" s="49" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="E187" s="47"/>
       <c r="F187" s="24" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="G187" s="25" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="H187" s="26"/>
       <c r="I187" s="27"/>
       <c r="J187" s="28"/>
       <c r="K187" s="29" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="L187" s="30"/>
       <c r="M187" s="31"/>
@@ -11745,7 +11745,7 @@
         <v>178</v>
       </c>
       <c r="R187" s="35" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="S187" s="52">
         <v>0.45800000000000002</v>
@@ -11761,20 +11761,20 @@
       </c>
       <c r="C188" s="33"/>
       <c r="D188" s="49" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="E188" s="47"/>
       <c r="F188" s="24" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="G188" s="25" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="H188" s="26"/>
       <c r="I188" s="27"/>
       <c r="J188" s="28"/>
       <c r="K188" s="29" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="L188" s="30"/>
       <c r="M188" s="31"/>
@@ -11785,7 +11785,7 @@
         <v>178</v>
       </c>
       <c r="R188" s="35" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="S188" s="52">
         <v>0.45800000000000002</v>
@@ -11801,20 +11801,20 @@
       </c>
       <c r="C189" s="33"/>
       <c r="D189" s="49" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="E189" s="47"/>
       <c r="F189" s="24" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="G189" s="25" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="H189" s="26"/>
       <c r="I189" s="27"/>
       <c r="J189" s="28"/>
       <c r="K189" s="29" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="L189" s="30"/>
       <c r="M189" s="31"/>
@@ -11822,10 +11822,10 @@
       <c r="O189" s="24"/>
       <c r="P189" s="33"/>
       <c r="Q189" s="34" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="R189" s="35" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="S189" s="36"/>
       <c r="T189" s="37"/>
@@ -11838,21 +11838,21 @@
         <v>397</v>
       </c>
       <c r="C190" s="33" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="D190" s="142"/>
       <c r="E190" s="47"/>
       <c r="F190" s="24" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="G190" s="25" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="H190" s="26"/>
       <c r="I190" s="27"/>
       <c r="J190" s="28"/>
       <c r="K190" s="29" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="L190" s="30"/>
       <c r="M190" s="31"/>
@@ -11874,23 +11874,23 @@
         <v>398</v>
       </c>
       <c r="C191" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D191" s="49" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="E191" s="47"/>
       <c r="F191" s="24" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="G191" s="25" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="H191" s="26"/>
       <c r="I191" s="27"/>
       <c r="J191" s="28"/>
       <c r="K191" s="29" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="L191" s="30"/>
       <c r="M191" s="31"/>
@@ -11912,23 +11912,23 @@
         <v>399</v>
       </c>
       <c r="C192" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D192" s="142" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="E192" s="47"/>
       <c r="F192" s="24" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="G192" s="25" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="H192" s="26"/>
       <c r="I192" s="27"/>
       <c r="J192" s="28"/>
       <c r="K192" s="29" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="L192" s="30"/>
       <c r="M192" s="31"/>
@@ -11951,27 +11951,27 @@
       </c>
       <c r="C193" s="33"/>
       <c r="D193" s="49" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="E193" s="47"/>
       <c r="F193" s="24" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="G193" s="25" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="H193" s="26"/>
       <c r="I193" s="27"/>
       <c r="J193" s="28"/>
       <c r="K193" s="29" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="L193" s="30"/>
       <c r="M193" s="31" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="N193" s="32" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="O193" s="24"/>
       <c r="P193" s="33"/>
@@ -11979,7 +11979,7 @@
         <v>178</v>
       </c>
       <c r="R193" s="35" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="S193" s="52">
         <v>1.42</v>
@@ -11995,20 +11995,20 @@
       </c>
       <c r="C194" s="33"/>
       <c r="D194" s="49" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="E194" s="47"/>
       <c r="F194" s="24" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="G194" s="25" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="H194" s="26"/>
       <c r="I194" s="27"/>
       <c r="J194" s="28"/>
       <c r="K194" s="29" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="L194" s="30"/>
       <c r="M194" s="31"/>
@@ -12019,7 +12019,7 @@
         <v>178</v>
       </c>
       <c r="R194" s="35" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="S194" s="52">
         <v>16.75</v>
@@ -12034,23 +12034,23 @@
         <v>402</v>
       </c>
       <c r="C195" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D195" s="142" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="E195" s="47"/>
       <c r="F195" s="24" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="G195" s="25" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="H195" s="26"/>
       <c r="I195" s="27"/>
       <c r="J195" s="28"/>
       <c r="K195" s="29" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="L195" s="30"/>
       <c r="M195" s="31"/>
@@ -12073,27 +12073,27 @@
       </c>
       <c r="C196" s="33"/>
       <c r="D196" s="49" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="E196" s="47"/>
       <c r="F196" s="24" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="G196" s="25" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="H196" s="26"/>
       <c r="I196" s="27"/>
       <c r="J196" s="28"/>
       <c r="K196" s="29" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="L196" s="30"/>
       <c r="M196" s="31" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="N196" s="32" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="O196" s="24"/>
       <c r="P196" s="33"/>
@@ -12101,7 +12101,7 @@
         <v>178</v>
       </c>
       <c r="R196" s="35" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="S196" s="52">
         <v>1.42</v>
@@ -12116,23 +12116,23 @@
         <v>404</v>
       </c>
       <c r="C197" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D197" s="49" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="E197" s="47"/>
       <c r="F197" s="24" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="G197" s="25" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="H197" s="26"/>
       <c r="I197" s="27"/>
       <c r="J197" s="28"/>
       <c r="K197" s="29" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="L197" s="30"/>
       <c r="M197" s="31"/>
@@ -12144,7 +12144,7 @@
       </c>
       <c r="R197" s="35"/>
       <c r="S197" s="36" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="T197" s="37"/>
       <c r="U197" s="38"/>
@@ -12156,23 +12156,23 @@
         <v>405</v>
       </c>
       <c r="C198" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D198" s="49" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="E198" s="47"/>
       <c r="F198" s="24" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="G198" s="25" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="H198" s="26"/>
       <c r="I198" s="27"/>
       <c r="J198" s="28"/>
       <c r="K198" s="29" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="L198" s="30"/>
       <c r="M198" s="31"/>
@@ -12184,7 +12184,7 @@
       </c>
       <c r="R198" s="35"/>
       <c r="S198" s="36" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="T198" s="37"/>
       <c r="U198" s="38"/>
@@ -12196,23 +12196,23 @@
         <v>406</v>
       </c>
       <c r="C199" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D199" s="49" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="E199" s="47"/>
       <c r="F199" s="24" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="G199" s="25" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="H199" s="26"/>
       <c r="I199" s="27"/>
       <c r="J199" s="28"/>
       <c r="K199" s="29" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="L199" s="30"/>
       <c r="M199" s="31"/>
@@ -12224,7 +12224,7 @@
       </c>
       <c r="R199" s="35"/>
       <c r="S199" s="36" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="T199" s="37"/>
       <c r="U199" s="38"/>
@@ -12236,23 +12236,23 @@
         <v>407</v>
       </c>
       <c r="C200" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D200" s="49" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="E200" s="47"/>
       <c r="F200" s="24" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="G200" s="25" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="H200" s="26"/>
       <c r="I200" s="27"/>
       <c r="J200" s="28"/>
       <c r="K200" s="29" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="L200" s="30"/>
       <c r="M200" s="31"/>
@@ -12264,7 +12264,7 @@
       </c>
       <c r="R200" s="35"/>
       <c r="S200" s="36" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="T200" s="37"/>
       <c r="U200" s="38"/>
@@ -12277,20 +12277,20 @@
       </c>
       <c r="C201" s="33"/>
       <c r="D201" s="49" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="E201" s="47"/>
       <c r="F201" s="24" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="G201" s="25" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="H201" s="26"/>
       <c r="I201" s="27"/>
       <c r="J201" s="28"/>
       <c r="K201" s="29" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="L201" s="30"/>
       <c r="M201" s="31"/>
@@ -12301,7 +12301,7 @@
         <v>178</v>
       </c>
       <c r="R201" s="35" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="S201" s="52">
         <v>16.75</v>
@@ -12316,23 +12316,23 @@
         <v>409</v>
       </c>
       <c r="C202" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D202" s="49" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="E202" s="47"/>
       <c r="F202" s="24" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="G202" s="25" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="H202" s="26"/>
       <c r="I202" s="27"/>
       <c r="J202" s="28"/>
       <c r="K202" s="29" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="L202" s="30"/>
       <c r="M202" s="31"/>
@@ -12344,7 +12344,7 @@
       </c>
       <c r="R202" s="35"/>
       <c r="S202" s="36" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="T202" s="37"/>
       <c r="U202" s="38"/>
@@ -12356,23 +12356,23 @@
         <v>410</v>
       </c>
       <c r="C203" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D203" s="49" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="E203" s="47"/>
       <c r="F203" s="24" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="G203" s="25" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="H203" s="26"/>
       <c r="I203" s="27"/>
       <c r="J203" s="28"/>
       <c r="K203" s="29" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="L203" s="30"/>
       <c r="M203" s="31"/>
@@ -12384,7 +12384,7 @@
       </c>
       <c r="R203" s="35"/>
       <c r="S203" s="36" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="T203" s="37"/>
       <c r="U203" s="38"/>
@@ -12396,23 +12396,23 @@
         <v>411</v>
       </c>
       <c r="C204" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D204" s="49" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="E204" s="47"/>
       <c r="F204" s="24" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="G204" s="25" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="H204" s="26"/>
       <c r="I204" s="27"/>
       <c r="J204" s="28"/>
       <c r="K204" s="29" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="L204" s="30"/>
       <c r="M204" s="31"/>
@@ -12424,7 +12424,7 @@
       </c>
       <c r="R204" s="35"/>
       <c r="S204" s="36" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="T204" s="37"/>
       <c r="U204" s="38"/>
@@ -12436,23 +12436,23 @@
         <v>412</v>
       </c>
       <c r="C205" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D205" s="49" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="E205" s="47"/>
       <c r="F205" s="24" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="G205" s="25" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="H205" s="26"/>
       <c r="I205" s="27"/>
       <c r="J205" s="28"/>
       <c r="K205" s="29" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="L205" s="30"/>
       <c r="M205" s="31"/>
@@ -12464,7 +12464,7 @@
       </c>
       <c r="R205" s="35"/>
       <c r="S205" s="36" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="T205" s="37"/>
       <c r="U205" s="38"/>
@@ -12476,21 +12476,21 @@
         <v>413</v>
       </c>
       <c r="C206" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D206" s="142"/>
       <c r="E206" s="47"/>
       <c r="F206" s="24" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="G206" s="25" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="H206" s="26"/>
       <c r="I206" s="27"/>
       <c r="J206" s="28"/>
       <c r="K206" s="29" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="L206" s="30"/>
       <c r="M206" s="31"/>
@@ -12513,27 +12513,27 @@
       </c>
       <c r="C207" s="33"/>
       <c r="D207" s="49" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="E207" s="47"/>
       <c r="F207" s="24" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="G207" s="25" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="H207" s="26"/>
       <c r="I207" s="27"/>
       <c r="J207" s="28"/>
       <c r="K207" s="29" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="L207" s="30"/>
       <c r="M207" s="31" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="N207" s="32" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="O207" s="24"/>
       <c r="P207" s="33"/>
@@ -12541,7 +12541,7 @@
         <v>178</v>
       </c>
       <c r="R207" s="35" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="S207" s="52">
         <v>1.42</v>
@@ -12556,23 +12556,23 @@
         <v>415</v>
       </c>
       <c r="C208" s="33" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D208" s="142" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="E208" s="47"/>
       <c r="F208" s="24" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="G208" s="25" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="H208" s="26"/>
       <c r="I208" s="27"/>
       <c r="J208" s="28"/>
       <c r="K208" s="29" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="L208" s="30"/>
       <c r="M208" s="31"/>
@@ -12595,20 +12595,20 @@
       </c>
       <c r="C209" s="33"/>
       <c r="D209" s="49" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="E209" s="47"/>
       <c r="F209" s="24" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="G209" s="25" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="H209" s="26"/>
       <c r="I209" s="27"/>
       <c r="J209" s="28"/>
       <c r="K209" s="29" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="L209" s="30"/>
       <c r="M209" s="31"/>
@@ -12619,7 +12619,7 @@
         <v>178</v>
       </c>
       <c r="R209" s="35" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="S209" s="52">
         <v>16.75</v>
@@ -12635,16 +12635,16 @@
       </c>
       <c r="C210" s="185"/>
       <c r="D210" s="49" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="E210" s="47" t="s">
         <v>43</v>
       </c>
       <c r="F210" s="155" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="G210" s="25" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="H210" s="26"/>
       <c r="I210" s="27">
@@ -12652,7 +12652,7 @@
       </c>
       <c r="J210" s="28"/>
       <c r="K210" s="29" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="L210" s="30"/>
       <c r="M210" s="31"/>
@@ -12663,7 +12663,7 @@
         <v>178</v>
       </c>
       <c r="R210" s="35" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="S210" s="52">
         <v>6.86</v>
@@ -12682,16 +12682,16 @@
       </c>
       <c r="C211" s="185"/>
       <c r="D211" s="49" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="E211" s="47" t="s">
         <v>43</v>
       </c>
       <c r="F211" s="155" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="G211" s="25" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="H211" s="26"/>
       <c r="I211" s="27">
@@ -12699,7 +12699,7 @@
       </c>
       <c r="J211" s="28"/>
       <c r="K211" s="29" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="L211" s="30"/>
       <c r="M211" s="31"/>
@@ -12710,7 +12710,7 @@
         <v>178</v>
       </c>
       <c r="R211" s="35" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="S211" s="52">
         <v>6.86</v>
@@ -12729,20 +12729,20 @@
       </c>
       <c r="C212" s="33"/>
       <c r="D212" s="49" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="E212" s="47"/>
       <c r="F212" s="24" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="G212" s="25" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="H212" s="26"/>
       <c r="I212" s="27"/>
       <c r="J212" s="28"/>
       <c r="K212" s="29" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="L212" s="30"/>
       <c r="M212" s="31"/>
@@ -12753,7 +12753,7 @@
         <v>178</v>
       </c>
       <c r="R212" s="35" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="S212" s="36"/>
       <c r="T212" s="37"/>
@@ -12767,20 +12767,20 @@
       </c>
       <c r="C213" s="33"/>
       <c r="D213" s="49" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="E213" s="47"/>
       <c r="F213" s="24" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="G213" s="25" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="H213" s="26"/>
       <c r="I213" s="27"/>
       <c r="J213" s="28"/>
       <c r="K213" s="29" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="L213" s="30"/>
       <c r="M213" s="31"/>
@@ -12791,7 +12791,7 @@
         <v>178</v>
       </c>
       <c r="R213" s="35" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="S213" s="36"/>
       <c r="T213" s="37"/>
@@ -12804,21 +12804,21 @@
         <v>421</v>
       </c>
       <c r="C214" s="33" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="D214" s="142"/>
       <c r="E214" s="47"/>
       <c r="F214" s="24" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="G214" s="25" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="H214" s="26"/>
       <c r="I214" s="27"/>
       <c r="J214" s="28"/>
       <c r="K214" s="29" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="L214" s="30"/>
       <c r="M214" s="31"/>
@@ -12841,16 +12841,16 @@
       </c>
       <c r="C215" s="185"/>
       <c r="D215" s="49" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="E215" s="47" t="s">
         <v>43</v>
       </c>
       <c r="F215" s="155" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="G215" s="25" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="H215" s="26"/>
       <c r="I215" s="27">
@@ -12858,7 +12858,7 @@
       </c>
       <c r="J215" s="28"/>
       <c r="K215" s="29" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="L215" s="30"/>
       <c r="M215" s="31"/>
@@ -12869,7 +12869,7 @@
         <v>178</v>
       </c>
       <c r="R215" s="35" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="S215" s="52">
         <v>6.86</v>
@@ -12888,16 +12888,16 @@
       </c>
       <c r="C216" s="185"/>
       <c r="D216" s="49" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="E216" s="47" t="s">
         <v>43</v>
       </c>
       <c r="F216" s="155" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="G216" s="25" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="H216" s="26"/>
       <c r="I216" s="27">
@@ -12905,7 +12905,7 @@
       </c>
       <c r="J216" s="28"/>
       <c r="K216" s="29" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="L216" s="30"/>
       <c r="M216" s="31"/>
@@ -12916,7 +12916,7 @@
         <v>178</v>
       </c>
       <c r="R216" s="35" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="S216" s="52">
         <v>6.86</v>

</xml_diff>